<commit_message>
added #2 for LastUpload in  Notes in Excel
</commit_message>
<xml_diff>
--- a/api/templates/pk_xpert_site_summary_site_wise_report/en.xlsx
+++ b/api/templates/pk_xpert_site_summary_site_wise_report/en.xlsx
@@ -29,16 +29,69 @@
     <t>Dates: &lt;Dates&gt;</t>
   </si>
   <si>
+    <t>&lt;StatesLabel&gt;: &lt;States&gt;</t>
+  </si>
+  <si>
+    <t>&lt;LgasLabel&gt;: &lt;Lgas&gt;</t>
+  </si>
+  <si>
+    <t>&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
+  </si>
+  <si>
+    <t>&lt;AssaysLabel&gt;: &lt;Assays&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Table&gt;</t>
+  </si>
+  <si>
+    <t>Last Upload</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>&lt;lastUploadOn&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalXpertTests&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalOtherTests&gt;</t>
+  </si>
+  <si>
+    <t>Xpert Site Summary Report - Site Wise</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>District</t>
+  </si>
+  <si>
+    <t>&lt;stateName&gt;</t>
+  </si>
+  <si>
+    <t>&lt;districtName&gt;</t>
+  </si>
+  <si>
+    <t>Province</t>
+  </si>
+  <si>
+    <t>Implementing Partner</t>
+  </si>
+  <si>
+    <t>&lt;implementingPartner&gt;</t>
+  </si>
+  <si>
+    <t>&lt;siteName&gt;</t>
+  </si>
+  <si>
     <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
       <t xml:space="preserve">Notes
-</t>
+1. </t>
     </r>
     <r>
       <rPr>
@@ -49,68 +102,9 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t>The result categories are represented by all the possible result combinations that GeneXpert sends to Aspect. For example, MTB Detected does not include MTB Detected Rif Detected, as they are considered different results</t>
+      <t>The result categories are represented by all the possible result combinations that GeneXpert sends to Aspect. For example, MTB Detected does not include MTB Detected Rif Detected, as they are considered different results.
+2. The Last Upload column shows the date when the last result of the site was performed</t>
     </r>
-  </si>
-  <si>
-    <t>&lt;StatesLabel&gt;: &lt;States&gt;</t>
-  </si>
-  <si>
-    <t>&lt;LgasLabel&gt;: &lt;Lgas&gt;</t>
-  </si>
-  <si>
-    <t>&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
-  </si>
-  <si>
-    <t>&lt;AssaysLabel&gt;: &lt;Assays&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Table&gt;</t>
-  </si>
-  <si>
-    <t>Last Upload</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>&lt;lastUploadOn&gt;</t>
-  </si>
-  <si>
-    <t>&lt;totalXpertTests&gt;</t>
-  </si>
-  <si>
-    <t>&lt;totalOtherTests&gt;</t>
-  </si>
-  <si>
-    <t>Xpert Site Summary Report - Site Wise</t>
-  </si>
-  <si>
-    <t>Site</t>
-  </si>
-  <si>
-    <t>District</t>
-  </si>
-  <si>
-    <t>&lt;stateName&gt;</t>
-  </si>
-  <si>
-    <t>&lt;districtName&gt;</t>
-  </si>
-  <si>
-    <t>Province</t>
-  </si>
-  <si>
-    <t>Implementing Partner</t>
-  </si>
-  <si>
-    <t>&lt;implementingPartner&gt;</t>
-  </si>
-  <si>
-    <t>&lt;siteName&gt;</t>
   </si>
 </sst>
 </file>
@@ -663,7 +657,7 @@
   <sheetData>
     <row r="1" spans="1:1011" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="3"/>
@@ -675,14 +669,17 @@
         <v>0</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="G2" s="21"/>
       <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="3" spans="1:1011" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="19"/>
       <c r="D3" s="19"/>
@@ -690,37 +687,49 @@
       <c r="F3" s="21"/>
       <c r="G3" s="21"/>
       <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
     </row>
     <row r="4" spans="1:1011" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" s="21"/>
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
     </row>
     <row r="5" spans="1:1011" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" s="21"/>
       <c r="G5" s="21"/>
       <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
     </row>
     <row r="6" spans="1:1011" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" s="21"/>
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
     </row>
     <row r="7" spans="1:1011" ht="57.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:1011" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -728,48 +737,48 @@
     </row>
     <row r="9" spans="1:1011" s="8" customFormat="1" ht="67.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="D9" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>19</v>
-      </c>
       <c r="E9" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="18" t="s">
         <v>8</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:1011" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>17</v>
-      </c>
       <c r="D10" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E10" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="G10" s="9" t="s">
         <v>11</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>12</v>
       </c>
       <c r="ALL10"/>
       <c r="ALM10"/>
@@ -786,7 +795,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="C3:E3"/>
-    <mergeCell ref="F2:H6"/>
+    <mergeCell ref="F2:K6"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>